<commit_message>
docs: update a table of requirements contradictions
</commit_message>
<xml_diff>
--- a/01_Анализ_требований/01_Таблица противоречий.xlsx
+++ b/01_Анализ_требований/01_Таблица противоречий.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="38">
   <si>
     <t>№
 пункта ТЗ</t>
@@ -47,9 +47,6 @@
     <t>Логическое противоречие</t>
   </si>
   <si>
-    <t>Переформулировать п.2: ...минимальное значение 1, но при уменьшении до 0 товар удаляется</t>
-  </si>
-  <si>
     <t>7, 13</t>
   </si>
   <si>
@@ -58,9 +55,6 @@
   </si>
   <si>
     <t>п. 7 конфликтует с п.13</t>
-  </si>
-  <si>
-    <t>Выбрать одну стратегию (рекомендовать фиксацию)</t>
   </si>
   <si>
     <t>1, 3, 4</t>
@@ -125,20 +119,32 @@
     <t>Избыточность</t>
   </si>
   <si>
-    <t>Убрать или переформулировать "Корзина поддерживает разный ассортимент"</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>На странице корзины отображается список товаров, их количество, цена за единицу и общая стоимость позиции.</t>
-  </si>
-  <si>
-    <t>нет</t>
-  </si>
-  <si>
     <t>п. 2 противоречит п.9
 Изменение количества до 0 (п.9) противоречит "не менее, чем до 1-го" п. 2</t>
+  </si>
+  <si>
+    <t>Исключить как избыточный</t>
+  </si>
+  <si>
+    <t>Переформулировать п.2: "...минимальное значение 1. Если пользователь уменьшает количество до 0, товар автоматически удаляется из корзин" и убрать п. 9 - будет поглощен</t>
+  </si>
+  <si>
+    <t>Выбрать одну стратегию (рекомендовать фиксацию для защиты покупателя от неожиданного повышения цен во время выбора)</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>В нумерации пропущен п.12.</t>
+  </si>
+  <si>
+    <t>Отсуствует пункт 12 - возможно потеря требования или ошибка в нумерации</t>
+  </si>
+  <si>
+    <t>Оформление</t>
+  </si>
+  <si>
+    <t>Уточнить у автора, должно ли быть требование на этом месте</t>
   </si>
 </sst>
 </file>
@@ -211,22 +217,6 @@
   </cellStyles>
   <dxfs count="4">
     <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF356854"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF356854"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF356854"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF356854"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF6F8F9"/>
@@ -250,13 +240,29 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF356854"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF356854"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF356854"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF356854"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="1">
     <tableStyle name="Лист1-style" pivot="0" count="4">
-      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
-      <tableStyleElement type="headerRow" dxfId="3"/>
-      <tableStyleElement type="firstRowStripe" dxfId="2"/>
-      <tableStyleElement type="secondRowStripe" dxfId="1"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="3"/>
+      <tableStyleElement type="headerRow" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="secondRowStripe" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -276,6 +282,10 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Таблица_противоречий" displayName="Таблица_противоречий" ref="A2:E9">
+  <autoFilter ref="A2:E9"/>
+  <sortState ref="A3:E9">
+    <sortCondition ref="D2:D9"/>
+  </sortState>
   <tableColumns count="5">
     <tableColumn id="1" name="№_x000a_пункта ТЗ"/>
     <tableColumn id="2" name="Текст пункта"/>
@@ -519,120 +529,124 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="102" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A3" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="102" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="89.25" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>10</v>
-      </c>
       <c r="C4" s="5" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>7</v>
       </c>
       <c r="E4" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="89.25" x14ac:dyDescent="0.2">
+      <c r="A5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="178.5" x14ac:dyDescent="0.2">
+      <c r="A6" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="178.5" x14ac:dyDescent="0.2">
-      <c r="A5" s="6" t="s">
+      <c r="C6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="D6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="E6" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="5" t="s">
+    </row>
+    <row r="7" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A7" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="B7" s="5" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A6" s="6" t="s">
+      <c r="C7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="D7" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="E7" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="5" t="s">
+    </row>
+    <row r="8" spans="1:5" ht="216.75" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="B8" s="5" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="216.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="D8" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>24</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A8" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
+        <v>35</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="10" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A10" s="8"/>

</xml_diff>